<commit_message>
Make the documents simpler: no cover page, plain black and grey style, shorter text with examples
</commit_message>
<xml_diff>
--- a/docs/04_Source_Target_Mapping.xlsx
+++ b/docs/04_Source_Target_Mapping.xlsx
@@ -43,18 +43,18 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="001F4E79"/>
+      <color rgb="00000000"/>
       <sz val="14"/>
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="001B2733"/>
+      <color rgb="00000000"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="001F4E79"/>
+      <color rgb="00000000"/>
       <sz val="11"/>
     </font>
     <font>
@@ -70,7 +70,7 @@
     <font>
       <name val="Arial"/>
       <i val="1"/>
-      <color rgb="0044546A"/>
+      <color rgb="00595959"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -83,12 +83,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F4E79"/>
+        <fgColor rgb="00404040"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EEF3F8"/>
+        <fgColor rgb="00F2F2F2"/>
       </patternFill>
     </fill>
   </fills>
@@ -102,16 +102,16 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00C9D2DC"/>
+        <color rgb="00BFBFBF"/>
       </left>
       <right style="thin">
-        <color rgb="00C9D2DC"/>
+        <color rgb="00BFBFBF"/>
       </right>
       <top style="thin">
-        <color rgb="00C9D2DC"/>
+        <color rgb="00BFBFBF"/>
       </top>
       <bottom style="thin">
-        <color rgb="00C9D2DC"/>
+        <color rgb="00BFBFBF"/>
       </bottom>
     </border>
   </borders>
@@ -507,14 +507,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>B2B Data Warehouse - Source-to-Target Mapping</t>
+          <t>Source-to-Target Mapping</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Version 1.0   |   22 October 2026   |   Author: Ali-Debugs</t>
+          <t>This workbook shows where every warehouse column comes from and which rule makes it.</t>
         </is>
       </c>
     </row>
@@ -524,56 +524,56 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>What this workbook holds</t>
+          <t>The sheets</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Source to Target - every column of staging, dw and mart: where it comes from and the rule that makes it.</t>
+          <t>Source to Target: every column of staging, dw and mart, with its source column and its rule.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Raw Copy - the raw layer: an exact, all-text copy of each source column.</t>
+          <t>Raw Copy: the raw layer, an exact copy of each source column, all as text.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Reject Rules - every staging rule that refuses a row, in the order it is checked, with the count in a fresh build.</t>
+          <t>Reject Rules: every rule that refuses a bad row, and how many rows it refused.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Data Dictionary - every column of the source and of the warehouse, with its type and meaning.</t>
+          <t>Data Dictionary: every column of the source and of the warehouse, with its type and meaning.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Lineage - for each report, the path from the dashboard back to the source.</t>
+          <t>Lineage: for each report, the path from the dashboard back to the source.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>History - the dimensions that keep history (SCD type 2) and how.</t>
+          <t>History: the tables that keep old versions (SCD type 2), and how.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Load Order - the 35 pipeline steps in the order run.py runs them.</t>
+          <t>Load Order: the 36 pipeline steps, in the order run.py runs them.</t>
         </is>
       </c>
     </row>
@@ -583,28 +583,28 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>How to read it</t>
+          <t>Good to know</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Layers: raw (exact copy) -&gt; staging (checked, typed) -&gt; dw (star schema) -&gt; mart (report views).</t>
+          <t>The data moves through four layers: raw (exact copy) -&gt; staging (checked) -&gt; dw (star schema) -&gt; mart (reports).</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Counts are from a fresh rebuild (fixed seed 42). Monthly figures depend on the build date; counts do not.</t>
+          <t>A bad row is never deleted. It is saved in etl.rejected_rows with the reason.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>A refused row is never dropped: it goes to etl.rejected_rows with the step and the reason.</t>
+          <t>Row counts come from a fresh build with the fixed seed 42. Monthly sales change with the build date; counts do not.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Give fact_logins a primary key (username, login_time), with migration 004
</commit_message>
<xml_diff>
--- a/docs/04_Source_Target_Mapping.xlsx
+++ b/docs/04_Source_Target_Mapping.xlsx
@@ -4456,7 +4456,11 @@
           <t>As is</t>
         </is>
       </c>
-      <c r="J83" s="6" t="inlineStr"/>
+      <c r="J83" s="6" t="inlineStr">
+        <is>
+          <t>Primary key with login_time</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="5" t="n">

</xml_diff>

<commit_message>
Docs: correct column meanings in dim_date, dim_company and the fact keys
</commit_message>
<xml_diff>
--- a/docs/04_Source_Target_Mapping.xlsx
+++ b/docs/04_Source_Target_Mapping.xlsx
@@ -9007,7 +9007,7 @@
       </c>
       <c r="F42" s="5" t="inlineStr">
         <is>
-          <t>Two-letter country code ('XX' = unknown)</t>
+          <t>Country where the company is registered</t>
         </is>
       </c>
     </row>
@@ -9231,7 +9231,7 @@
       </c>
       <c r="F49" s="6" t="inlineStr">
         <is>
-          <t>Day as a number YYYYMMDD; points to dim_date</t>
+          <t>The day as a number YYYYMMDD, for example 20261022</t>
         </is>
       </c>
     </row>
@@ -9327,7 +9327,7 @@
       </c>
       <c r="F52" s="5" t="inlineStr">
         <is>
-          <t>First day of the month</t>
+          <t>Month number (1-12)</t>
         </is>
       </c>
     </row>
@@ -9647,7 +9647,7 @@
       </c>
       <c r="F62" s="5" t="inlineStr">
         <is>
-          <t>Source company id</t>
+          <t>Source id of the company that serves this person</t>
         </is>
       </c>
     </row>
@@ -10159,7 +10159,7 @@
       </c>
       <c r="F78" s="5" t="inlineStr">
         <is>
-          <t>Warehouse key of one company version (surrogate key)</t>
+          <t>The company version valid on the login day (points to dim_company)</t>
         </is>
       </c>
     </row>
@@ -10191,7 +10191,7 @@
       </c>
       <c r="F79" s="6" t="inlineStr">
         <is>
-          <t>Warehouse key of a device kind</t>
+          <t>The device of the visit (points to dim_device)</t>
         </is>
       </c>
     </row>
@@ -10223,7 +10223,7 @@
       </c>
       <c r="F80" s="5" t="inlineStr">
         <is>
-          <t>Two-letter country code ('XX' = unknown)</t>
+          <t>Country of the visitor's IP address ('XX' = not in the lookup file); points to dim_country</t>
         </is>
       </c>
     </row>
@@ -10351,7 +10351,7 @@
       </c>
       <c r="F84" s="5" t="inlineStr">
         <is>
-          <t>Warehouse key of one company version (surrogate key)</t>
+          <t>The company version valid on the order day (points to dim_company)</t>
         </is>
       </c>
     </row>
@@ -10383,7 +10383,7 @@
       </c>
       <c r="F85" s="6" t="inlineStr">
         <is>
-          <t>Warehouse key of one end-customer version (surrogate key)</t>
+          <t>The end-customer version valid on the order day (points to dim_end_customer)</t>
         </is>
       </c>
     </row>
@@ -10415,7 +10415,7 @@
       </c>
       <c r="F86" s="5" t="inlineStr">
         <is>
-          <t>Warehouse key of one product version (surrogate key)</t>
+          <t>The product version valid on the order day (points to dim_product)</t>
         </is>
       </c>
     </row>
@@ -12367,7 +12367,7 @@
       </c>
       <c r="F147" s="6" t="inlineStr">
         <is>
-          <t>Two-letter country code ('XX' = unknown)</t>
+          <t>Country where the company is registered</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mapping workbook: fix the order_date type and column meanings borrowed from other tables
</commit_message>
<xml_diff>
--- a/docs/04_Source_Target_Mapping.xlsx
+++ b/docs/04_Source_Target_Mapping.xlsx
@@ -1697,7 +1697,7 @@
       </c>
       <c r="E23" s="6" t="inlineStr">
         <is>
-          <t>timestamptz</t>
+          <t>timestamp</t>
         </is>
       </c>
       <c r="F23" s="6" t="inlineStr">
@@ -5960,7 +5960,7 @@
     <row r="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>The raw layer keeps every column as text, so no value can stop the copy. Orders and order items are refreshed by CDC in an incremental run.</t>
+          <t>The raw layer keeps every column as text, so no value can stop the copy. In an incremental run, orders and order items are refreshed by CDC and the web log gets only its new lines; the other tables are copied in full.</t>
         </is>
       </c>
     </row>
@@ -8581,7 +8581,7 @@
       </c>
       <c r="D29" s="6" t="inlineStr">
         <is>
-          <t>timestamptz</t>
+          <t>timestamp</t>
         </is>
       </c>
       <c r="E29" s="6" t="inlineStr">
@@ -11055,7 +11055,7 @@
       </c>
       <c r="F106" s="5" t="inlineStr">
         <is>
-          <t>running, success, failed or abandoned</t>
+          <t>running, success or failed</t>
         </is>
       </c>
     </row>
@@ -11439,7 +11439,7 @@
       </c>
       <c r="F118" s="5" t="inlineStr">
         <is>
-          <t>Country name</t>
+          <t>Country of the visitor's IP address ('Unknown' = not in the lookup file)</t>
         </is>
       </c>
     </row>
@@ -11727,7 +11727,7 @@
       </c>
       <c r="F127" s="6" t="inlineStr">
         <is>
-          <t>Country name</t>
+          <t>Country where the company is registered</t>
         </is>
       </c>
     </row>
@@ -12015,7 +12015,7 @@
       </c>
       <c r="F136" s="5" t="inlineStr">
         <is>
-          <t>Country name</t>
+          <t>The country with the most logins (from the IP address)</t>
         </is>
       </c>
     </row>
@@ -12335,7 +12335,7 @@
       </c>
       <c r="F146" s="5" t="inlineStr">
         <is>
-          <t>Company or product name</t>
+          <t>Company name</t>
         </is>
       </c>
     </row>
@@ -12805,7 +12805,7 @@
       </c>
       <c r="D161" s="6" t="inlineStr">
         <is>
-          <t>timestamptz</t>
+          <t>timestamp</t>
         </is>
       </c>
       <c r="E161" s="6" t="inlineStr">
@@ -12815,7 +12815,7 @@
       </c>
       <c r="F161" s="6" t="inlineStr">
         <is>
-          <t>Day of the order</t>
+          <t>Date and time of the order, in business time (Buenos Aires)</t>
         </is>
       </c>
     </row>
@@ -12911,7 +12911,7 @@
       </c>
       <c r="F164" s="5" t="inlineStr">
         <is>
-          <t>Company or product name</t>
+          <t>Product name</t>
         </is>
       </c>
     </row>
@@ -13039,7 +13039,7 @@
       </c>
       <c r="F168" s="5" t="inlineStr">
         <is>
-          <t>Time of the first page of the visit (with time zone)</t>
+          <t>Time of this log line (one page); fact_logins keeps the first line of each visit</t>
         </is>
       </c>
     </row>
@@ -13199,7 +13199,7 @@
       </c>
       <c r="F173" s="6" t="inlineStr">
         <is>
-          <t>Two-letter country code ('XX' = unknown)</t>
+          <t>Country of the IP address ('XX' = not in the lookup file)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Docs: fix review findings and explain the country outrigger
</commit_message>
<xml_diff>
--- a/docs/04_Source_Target_Mapping.xlsx
+++ b/docs/04_Source_Target_Mapping.xlsx
@@ -7698,7 +7698,7 @@
       <c r="D25" s="6" t="inlineStr"/>
       <c r="E25" s="6">
         <f>SUM(E4:E24)</f>
-        <v/>
+        <v>1228</v>
       </c>
     </row>
   </sheetData>
@@ -9007,7 +9007,7 @@
       </c>
       <c r="F42" s="5" t="inlineStr">
         <is>
-          <t>Country where the company is registered</t>
+          <t>Country where the company is registered; points to dim_country</t>
         </is>
       </c>
     </row>
@@ -13282,22 +13282,22 @@
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>dw.fact_logins, dw.dim_device</t>
+          <t>dw.fact_logins, dw.dim_date, dw.dim_company, dw.dim_device, dw.dim_country</t>
         </is>
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t>staging.stg_web_logs</t>
+          <t>staging.stg_web_logs, stg_companies</t>
         </is>
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>raw.raw_web_logs, raw.raw_users</t>
+          <t>raw.raw_web_logs, raw_users, raw_ip_country, raw_companies</t>
         </is>
       </c>
       <c r="G2" s="5" t="inlineStr">
         <is>
-          <t>access.log, b2b.users</t>
+          <t>access.log, ip_country.csv, b2b.users, b2b.companies</t>
         </is>
       </c>
     </row>
@@ -13319,22 +13319,22 @@
       </c>
       <c r="D3" s="6" t="inlineStr">
         <is>
-          <t>dw.fact_logins, dw.fact_sales, dw.dim_country, dw.dim_company, dw.dim_product</t>
+          <t>dw.fact_logins, dw.fact_sales, dw.dim_date, dw.dim_company, dw.dim_country, dw.dim_device, dw.dim_product, dw.dim_end_customer</t>
         </is>
       </c>
       <c r="E3" s="6" t="inlineStr">
         <is>
-          <t>staging.stg_web_logs, stg_orders, stg_order_items, stg_companies, stg_products</t>
+          <t>staging.stg_web_logs, stg_orders, stg_order_items, stg_companies, stg_suppliers, stg_products, stg_end_customers</t>
         </is>
       </c>
       <c r="F3" s="6" t="inlineStr">
         <is>
-          <t>raw.raw_web_logs, raw_ip_country, raw_orders, raw_order_items, raw_companies, raw_products</t>
+          <t>raw.raw_web_logs, raw_users, raw_ip_country, raw_orders, raw_order_items, raw_companies, raw_suppliers, raw_products, raw_end_customers</t>
         </is>
       </c>
       <c r="G3" s="6" t="inlineStr">
         <is>
-          <t>access.log, ip_country.csv, b2b.orders, b2b.order_items, b2b.companies, b2b.products</t>
+          <t>access.log, ip_country.csv, b2b.users, b2b.orders, b2b.order_items, b2b.companies, b2b.suppliers, b2b.products, b2b.end_customers</t>
         </is>
       </c>
     </row>
@@ -13356,22 +13356,22 @@
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>dw.fact_sales, dw.dim_date, dw.dim_company</t>
+          <t>dw.fact_sales, dw.dim_date, dw.dim_company, dw.dim_country, dw.dim_product, dw.dim_end_customer</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t>staging.stg_orders, stg_order_items</t>
+          <t>staging.stg_orders, stg_order_items, stg_companies, stg_suppliers, stg_products, stg_end_customers</t>
         </is>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>raw.raw_orders, raw.raw_order_items</t>
+          <t>raw.raw_orders, raw_order_items, raw_companies, raw_suppliers, raw_products, raw_end_customers, raw_ip_country</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>b2b.orders, b2b.order_items</t>
+          <t>b2b.orders, b2b.order_items, b2b.companies, b2b.suppliers, b2b.products, b2b.end_customers, ip_country.csv</t>
         </is>
       </c>
     </row>

</xml_diff>